<commit_message>
Expand automation workflows and ATT data repair
</commit_message>
<xml_diff>
--- a/config/templates/OAS-K_Configuration_Template v.1.xlsx
+++ b/config/templates/OAS-K_Configuration_Template v.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57B8CF6-50FC-49CB-9E08-78DC5FD8FFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996A95F4-DA66-4A3E-8D9E-6F9AAA58152F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="15" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" r:id="rId1"/>
@@ -30,8 +30,10 @@
     <sheet name="HRIS_Assisted_Steps" sheetId="15" r:id="rId15"/>
     <sheet name="Comparison_Settings" sheetId="16" r:id="rId16"/>
     <sheet name="Attachment_Consolidation" sheetId="17" r:id="rId17"/>
+    <sheet name="Att_Data_Repair" sheetId="18" r:id="rId18"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">Att_Data_Repair!$A$3:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">Attachment_Consolidation!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Attendance_Settings!$A$3:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Attendance_Sources!$A$3:$F$264</definedName>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15925" uniqueCount="6322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15981" uniqueCount="6350">
   <si>
     <t>Panduan Konfigurasi OAS-K</t>
   </si>
@@ -19057,6 +19059,90 @@
   </si>
   <si>
     <t>07-2026</t>
+  </si>
+  <si>
+    <t>Att Data Repair</t>
+  </si>
+  <si>
+    <t>enabled</t>
+  </si>
+  <si>
+    <t>Aktifkan modul Att Data Repair.</t>
+  </si>
+  <si>
+    <t>minimum_duration_minutes</t>
+  </si>
+  <si>
+    <t>Durasi minimum repair dalam menit.</t>
+  </si>
+  <si>
+    <t>weekday_default_in</t>
+  </si>
+  <si>
+    <t>09:30</t>
+  </si>
+  <si>
+    <t>Jam masuk default Senin-Jumat.</t>
+  </si>
+  <si>
+    <t>weekday_default_out</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>Jam keluar default Senin-Jumat.</t>
+  </si>
+  <si>
+    <t>saturday_default_in</t>
+  </si>
+  <si>
+    <t>Jam masuk default Sabtu.</t>
+  </si>
+  <si>
+    <t>saturday_default_out</t>
+  </si>
+  <si>
+    <t>12:05</t>
+  </si>
+  <si>
+    <t>Jam keluar default Sabtu.</t>
+  </si>
+  <si>
+    <t>sunday_invalid_default_in</t>
+  </si>
+  <si>
+    <t>Jam masuk default Minggu bila jam invalid.</t>
+  </si>
+  <si>
+    <t>sunday_invalid_default_out</t>
+  </si>
+  <si>
+    <t>Jam keluar default Minggu bila jam invalid.</t>
+  </si>
+  <si>
+    <t>txt_max_rows</t>
+  </si>
+  <si>
+    <t>Maksimum baris per TXT Att Data Repair.</t>
+  </si>
+  <si>
+    <t>generate_txt</t>
+  </si>
+  <si>
+    <t>Buat TXT HRIS.</t>
+  </si>
+  <si>
+    <t>generate_excel_report</t>
+  </si>
+  <si>
+    <t>Buat Excel report audit.</t>
+  </si>
+  <si>
+    <t>Gunakan periode global bila UI mendukung.</t>
+  </si>
+  <si>
+    <t>Gunakan output root global bila UI mendukung.</t>
   </si>
 </sst>
 </file>
@@ -19204,15 +19290,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -19595,7 +19681,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="14"/>
@@ -19833,7 +19919,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6142</v>
       </c>
       <c r="B1" s="14"/>
@@ -19841,7 +19927,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -19996,7 +20082,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6158</v>
       </c>
       <c r="B1" s="14"/>
@@ -20006,7 +20092,7 @@
       <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -21628,7 +21714,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6180</v>
       </c>
       <c r="B1" s="14"/>
@@ -21636,7 +21722,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -21698,7 +21784,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6182</v>
       </c>
       <c r="B1" s="14"/>
@@ -21706,7 +21792,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -22062,7 +22148,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6228</v>
       </c>
       <c r="B1" s="14"/>
@@ -22071,7 +22157,7 @@
       <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -24769,7 +24855,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6304</v>
       </c>
       <c r="B1" s="14"/>
@@ -24782,7 +24868,7 @@
       <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -26451,7 +26537,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6318</v>
       </c>
       <c r="B1" s="14"/>
@@ -26459,7 +26545,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -26535,7 +26621,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6319</v>
       </c>
       <c r="B1" s="14"/>
@@ -26543,7 +26629,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -26600,6 +26686,244 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih nilai dari daftar yang tersedia." promptTitle="OAS-K" prompt="Gunakan salah satu nilai yang tersedia." sqref="B4" xr:uid="{00000000-0002-0000-1000-000000000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8733B8-572A-4001-9EB4-23AFEAE5FE2D}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="24" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>6322</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="30" customHeight="1">
+      <c r="A2" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+    </row>
+    <row r="3" spans="1:4" ht="30" customHeight="1">
+      <c r="A3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16">
+      <c r="A4" s="6" t="s">
+        <v>6323</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6324</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16">
+      <c r="A5" s="6" t="s">
+        <v>6325</v>
+      </c>
+      <c r="B5" s="7">
+        <v>61</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>6326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16">
+      <c r="A6" s="6" t="s">
+        <v>6327</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>6328</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>6329</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16">
+      <c r="A7" s="6" t="s">
+        <v>6330</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>6331</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>6332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16">
+      <c r="A8" s="6" t="s">
+        <v>6333</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>6328</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>6334</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16">
+      <c r="A9" s="6" t="s">
+        <v>6335</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>6336</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>6337</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16">
+      <c r="A10" s="6" t="s">
+        <v>6338</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>6328</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>6339</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16">
+      <c r="A11" s="6" t="s">
+        <v>6340</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>6336</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>6341</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16">
+      <c r="A12" s="6" t="s">
+        <v>6342</v>
+      </c>
+      <c r="B12" s="7">
+        <v>10000</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>6343</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16">
+      <c r="A13" s="6" t="s">
+        <v>6344</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>6345</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16">
+      <c r="A14" s="6" t="s">
+        <v>6346</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>6347</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16">
+      <c r="A15" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>6348</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16">
+      <c r="A16" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>6349</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:D16" xr:uid="{00000000-0009-0000-0000-000011000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih nilai dari daftar yang tersedia." promptTitle="OAS-K" prompt="Gunakan salah satu nilai yang tersedia." sqref="B4 B13:B16" xr:uid="{8AFF7EC3-73DA-446C-8B5A-2878F3830617}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -26619,7 +26943,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="14"/>
@@ -26627,7 +26951,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -26712,7 +27036,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>69</v>
       </c>
       <c r="B1" s="14"/>
@@ -26720,7 +27044,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -26840,7 +27164,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>81</v>
       </c>
       <c r="B1" s="14"/>
@@ -26850,7 +27174,7 @@
       <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -32134,7 +32458,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>835</v>
       </c>
       <c r="B1" s="14"/>
@@ -32142,7 +32466,7 @@
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="14"/>
@@ -32445,7 +32769,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>877</v>
       </c>
       <c r="B1" s="14"/>
@@ -32458,7 +32782,7 @@
       <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -70408,7 +70732,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>5155</v>
       </c>
       <c r="B1" s="14"/>
@@ -70421,7 +70745,7 @@
       <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -77627,14 +77951,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6133</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>
@@ -77705,14 +78029,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>6137</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="14"/>

</xml_diff>